<commit_message>
Stabilize Daily Work Report layout and Section 5/6 structure
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/Material_Inventory.xlsx
+++ b/Na-aba/home/data/Material_Inventory.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S464"/>
+  <dimension ref="A1:S465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24247,6 +24247,59 @@
         <v>10</v>
       </c>
       <c r="S464" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>462</v>
+      </c>
+      <c r="B465" t="inlineStr"/>
+      <c r="C465" t="inlineStr"/>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>MT약품</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>자동등록</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+      <c r="K465" t="n">
+        <v>0</v>
+      </c>
+      <c r="L465" t="n">
+        <v>0</v>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr"/>
+      <c r="O465" t="inlineStr"/>
+      <c r="P465" t="inlineStr"/>
+      <c r="Q465" t="n">
+        <v>0</v>
+      </c>
+      <c r="R465" t="n">
+        <v>10</v>
+      </c>
+      <c r="S465" t="n">
         <v>1</v>
       </c>
     </row>
@@ -24261,7 +24314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24411,10 +24464,26 @@
           <t>K1-PJT</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -24427,6 +24496,273 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B3" t="n">
+        <v>405</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-100</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B4" t="n">
+        <v>408</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-100</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45778.88671622195</v>
+      </c>
+      <c r="B5" t="n">
+        <v>433</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감) (nan)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>45778.88671622195</v>
+      </c>
+      <c r="B6" t="n">
+        <v>434</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감) (nan)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B7" t="n">
+        <v>462</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>-20</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>K1-PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24500,7 +24836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CB2"/>
+  <dimension ref="A1:CB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24906,7 +25242,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -24920,13 +25256,9 @@
       <c r="D2" t="n">
         <v>100</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
-        <v>46147.34000990329</v>
+        <v>46147.34000990741</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -24994,66 +25326,48 @@
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AA2" t="n">
+        <v>0</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AD2" t="n">
+        <v>0</v>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AG2" t="n">
+        <v>0</v>
       </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AJ2" t="n">
+        <v>0</v>
       </c>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AM2" t="n">
+        <v>0</v>
       </c>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AP2" t="n">
+        <v>0</v>
       </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AS2" t="n">
+        <v>0</v>
       </c>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AV2" t="n">
+        <v>0</v>
       </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AY2" t="n">
+        <v>0</v>
       </c>
       <c r="AZ2" t="n">
         <v>0</v>
@@ -25096,11 +25410,7 @@
       <c r="BL2" t="n">
         <v>2</v>
       </c>
-      <c r="BM2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr">
         <is>
           <t>롯데건설</t>
@@ -25123,11 +25433,7 @@
           <t>ASME B31.3</t>
         </is>
       </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr">
         <is>
@@ -25135,7 +25441,625 @@
         </is>
       </c>
       <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr"/>
+      <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>405</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="1" t="n">
+        <v>46147.87794667824</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>R-RAY(Se-75)</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2550000</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>408</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="1" t="n">
+        <v>46147.87911841435</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>R-RAY(Se-75)</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>2550000</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>K1-PJT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>462</v>
+      </c>
+      <c r="D5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46147.88671621533</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>4300</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>86000</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>스타렉스91주8839</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>ASME B31.3</t>
+        </is>
+      </c>
+      <c r="BX5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: finalize Integrated-Smart-Manager-Final and Daily Usage layout restoration
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/Material_Inventory.xlsx
+++ b/Na-aba/home/data/Material_Inventory.xlsx
@@ -1,18 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DailyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Budget" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21717,11 +21715,7 @@
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
-      <c r="F413" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr"/>
       <c r="H413" t="inlineStr">
         <is>
@@ -23161,11 +23155,7 @@
         </is>
       </c>
       <c r="E443" t="inlineStr"/>
-      <c r="F443" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr"/>
       <c r="H443" t="inlineStr"/>
       <c r="I443" t="inlineStr"/>
@@ -23955,26 +23945,10 @@
           <t>K1-PJT</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -23994,67 +23968,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Material ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Usage</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Entry Date</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>MaterialID</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>EntryDate</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24644,630 +24557,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>LaborCost</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>MaterialCost</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>OutsourceCost</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>LaborDetail</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>MaterialDetail</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ExpenseDetail</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>UnitPrice</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Spec</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>이사</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
-        <v>55250000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>부장</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
-        <v>55250000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>차장</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>47670000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>과장</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="n">
-        <v>41170000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>대리</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
-        <v>37920000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>계장</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="n">
-        <v>34670000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>주임</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="n">
-        <v>31420000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Labor</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>기사</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="n">
-        <v>29250000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PT 약품</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>세척액</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>PT 약품</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>침투액</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PT 약품</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>현상액</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>MT 약품</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>자분페인트</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>2350</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>MT 약품</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>흑색자분</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>방사선투과검사 필름</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>MX125</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>매</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>990</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>글리세린</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>20L</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>통</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>필름 현상액</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>3L</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>통</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>16500</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>필름 정착액</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>3L</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>통</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>16500</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>수적방지액</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>200mL</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>통</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>차량유지비</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>주유, 수리, 통행, 주차 등</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>소모품비</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>장갑,일회용 작업복외</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>복리후생비</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>생수, 음료 외 기타</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>1666</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Expense</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Se-175</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>방사성동위원소 구매</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>35714</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Outsource</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>케이엔디이</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>방사선투과검사</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>공수</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>15000</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update NDT billing sync: Add location selection & align calculation logic
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/Material_Inventory.xlsx
+++ b/Na-aba/home/data/Material_Inventory.xlsx
@@ -21,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23927,7 +23930,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46185</v>
+        <v>46198</v>
       </c>
       <c r="B2" t="n">
         <v>409</v>
@@ -23942,35 +23945,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>의왕 주배관 현장 사용 (자동 차감)</t>
+          <t>가산~가평 현장 사용 (자동 차감)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>의왕 주배관</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>가산~가평</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -24046,7 +24033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM2"/>
+  <dimension ref="A1:CL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24500,19 +24487,14 @@
           <t>기술료</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
-        <is>
-          <t>수량</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46185</v>
+      <c r="A2" s="2" t="n">
+        <v>46198</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>의왕 주배관</t>
+          <t>가산~가평</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -24523,7 +24505,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
-        <v>46190.97575810185</v>
+        <v>46198.00841747563</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -24556,7 +24538,7 @@
         <v>25</v>
       </c>
       <c r="Q2" t="n">
-        <v>69810</v>
+        <v>132359</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -24565,7 +24547,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>1745243</v>
+        <v>3308975</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -24646,7 +24628,11 @@
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
       <c r="BW2" t="inlineStr"/>
       <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
@@ -24658,7 +24644,7 @@
       <c r="CA2" t="inlineStr"/>
       <c r="CB2" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>야간</t>
         </is>
       </c>
       <c r="CC2" t="inlineStr">
@@ -24683,16 +24669,13 @@
         <v>84475</v>
       </c>
       <c r="CJ2" t="n">
-        <v>871575</v>
+        <v>1692225</v>
       </c>
       <c r="CK2" t="n">
-        <v>697260</v>
+        <v>1353780</v>
       </c>
       <c r="CL2" t="n">
-        <v>91933</v>
-      </c>
-      <c r="CM2" t="n">
-        <v>0</v>
+        <v>178495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update NDT billing tab to itemize expenses, add liability deduction fee, and adjust Excel formatting
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/Material_Inventory.xlsx
+++ b/Na-aba/home/data/Material_Inventory.xlsx
@@ -21,11 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -56,10 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -21615,7 +21612,7 @@
         <v>10</v>
       </c>
       <c r="S410" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="411">
@@ -23941,7 +23938,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-25</v>
+        <v>-1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -23954,10 +23951,26 @@
           <t>가산~가평</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -24033,7 +24046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL2"/>
+  <dimension ref="A1:CM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24487,9 +24500,14 @@
           <t>기술료</t>
         </is>
       </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46198</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -24501,11 +24519,11 @@
         <v>409</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="1" t="n">
-        <v>46198.00841747563</v>
+        <v>46198.41365496528</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -24535,10 +24553,10 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>132359</v>
+        <v>125062</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -24547,7 +24565,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>3308975</v>
+        <v>125062</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -24630,10 +24648,14 @@
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr"/>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>KS B 0845</t>
+        </is>
+      </c>
       <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr">
@@ -24663,19 +24685,22 @@
         <v>1</v>
       </c>
       <c r="CH2" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="CI2" t="n">
-        <v>84475</v>
+        <v>3379</v>
       </c>
       <c r="CJ2" t="n">
-        <v>1692225</v>
+        <v>63860</v>
       </c>
       <c r="CK2" t="n">
-        <v>1353780</v>
+        <v>51088</v>
       </c>
       <c r="CL2" t="n">
-        <v>178495</v>
+        <v>6735</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update safety report automation: Fix duplicated text in HWP, support multiple image insertions with auto-adjustment, and optimize layouts
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/Material_Inventory.xlsx
+++ b/Na-aba/home/data/Material_Inventory.xlsx
@@ -21,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -54,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23805,7 +23801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23924,65 +23920,6 @@
           <t>수량</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B2" t="n">
-        <v>409</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>가산~가평 현장 사용 (자동 차감)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24046,7 +23983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM2"/>
+  <dimension ref="A1:CM1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24504,203 +24441,6 @@
         <is>
           <t>수량</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>409</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46198.41365496528</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>R-RAY(Se-75)</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>125062</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>125062</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>가스공사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>KS B 0845</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>매</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>야간</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>Ir-192 또는 Se-75 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>15mm 이하 (1.0)</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>3379</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>63860</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>51088</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>6735</v>
-      </c>
-      <c r="CM2" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>